<commit_message>
Drop C-tier from batch3: 87 -> 60 papers
Aligns batch3 with batch2's convention of not shipping C-tier candidates.
PDF names are numbered per tier (A001.., B001.., C001..), so removing every
C* file leaves the S/A/B filenames untouched -- the A001-A008 already pushed
stay valid.

The surviving 60 are all automation-level A with fully public benchmarks:
those two dimensions carry most of the repro-priority weight, so everything
that scored low on them had already fallen into C.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/batch3/信息抽取batch3.xlsx
+++ b/batch3/信息抽取batch3.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'batch3汇总'!$A$1:$W$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'batch3汇总'!$A$1:$W$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'字段说明'!$A$1:$B$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W88"/>
+  <dimension ref="A1:W61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6645,2686 +6645,8 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Base-resolution binding profile prediction of proteins on RNAs with deep learning.</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Nucleic Acids Research</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>蛋白与结构</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>ENCODE eCLIP-seq（225 套配对数据 / 150 个 RBP）</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>225 套 paired-end eCLIP-seq：K562 120 套、HepG2 103 套、肾上腺 2 套；HepG2 total RNA-seq 3 样本识别 17,364 个表达基因、polyA+ 10 样本识别 18,049 个</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>TIA1（ENST00000531983.1）与 HNRNPC（ENST00000559273.5）上 PCC 分别 0.91 与 0.79，优于对照；对照 RBPNet 仅用 HepG2 的 103 套训练，本方法用全部 225 套；以良性 SNP 平均突变效应 0.03 为阈值筛出 30,751 个致病 SNP</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>皮尔逊相关系数 PCC（预测结合谱 vs eCLIP 交联信号）、AUC；碱基分辨率</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1093/nar/gkaf748</t>
-        </is>
-      </c>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>★★★ ENCODE 数据完全公开可批量下载，PCC 为客观指标，是本批生信方向最易复现的一篇</t>
-        </is>
-      </c>
-      <c r="O62" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="P62" t="inlineStr">
-        <is>
-          <t>生信</t>
-        </is>
-      </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>蛋白与结构</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T62" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U62" t="n">
-        <v>65.09999999999999</v>
-      </c>
-      <c r="V62" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="W62" t="inlineStr">
-        <is>
-          <t>C001_Base-resolution binding profile prediction of proteins on RNAs with de.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Development and validation of a pre-trained language model for neonatal morbidities: a retrospective, multicentre, prognostic study.</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>The Lancet Digital Health</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>临床NLP与决策</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>（本批深读未取到文件，见复刻备注）</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>physionet.org/content/mimiciii/1.4/</t>
-        </is>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.landig.2025.100926</t>
-        </is>
-      </c>
-      <c r="N63" t="inlineStr">
-        <is>
-          <t>⚠️该 DOI 在 fulltext/ 与隔离区均未找到对应文件，需先补全文再抽取</t>
-        </is>
-      </c>
-      <c r="O63" t="n">
-        <v>23.8</v>
-      </c>
-      <c r="P63" t="inlineStr">
-        <is>
-          <t>数字医疗</t>
-        </is>
-      </c>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>临床NLP与决策</t>
-        </is>
-      </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S63" t="inlineStr">
-        <is>
-          <t>部分(仅排名或定性)</t>
-        </is>
-      </c>
-      <c r="T63" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U63" t="n">
-        <v>63.9</v>
-      </c>
-      <c r="V63" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W63" t="inlineStr">
-        <is>
-          <t>C002_Development and validation of a pre-trained language model for neonata.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Large-Scale Logo Detection.</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Logo4500（自建）· FoodLogoDet-1500 · LogoDet-3K · FlickrLogos-32</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Logo4500：293,298 图 / 426,221 个 logo 实例 / 4,500 类，人工逐实例标注，为目前最大公开 logo 数据集；FlickrLogos-32 为 32 类每类 70 图</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>FALDR-Net 达 AP 71.3% / AP50 91.0% / AP75 80.6% / APs 32.6% / APl 96.0%，几乎全面超越对照方法；作为预训练集的价值：TOOD 在 FoodLogoDet-1500 上 AP/AP50/AP75 +3.3%/3.9%/3.4%；ResNet-50 Top-1 识别 +6.1%（用 LogoDet-3K 仅 +1.6%）；VGG-16 Top-5 +5%（对照 +1.7%）；OW-DETR mAP +11.4%（对照仅 +0.3%）</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>AP / AP50 / AP75 / APs / APm / APl（IoU=0.5 分尺寸统计）、Top-1/Top-5 识别准确率</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3630505</t>
-        </is>
-      </c>
-      <c r="N64" t="inlineStr">
-        <is>
-          <t>★★★ 自称目前最大公开 logo 数据集，同时给检测与预训练迁移两类对比；⚠️ 未见下载链接，需向作者索取</t>
-        </is>
-      </c>
-      <c r="O64" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P64" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q64" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="R64" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S64" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T64" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U64" t="n">
-        <v>63</v>
-      </c>
-      <c r="V64" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W64" t="inlineStr">
-        <is>
-          <t>C003_Large-Scale Logo Detection.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>SpaceEra++: A Unified Framework Towards 3D Spatial Reasoning in Video.</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>ScanForgeQA（自建）· ScanNet 系列 3D 空间推理评测</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>扫描视频常达数千帧而现有 VLM 只能吃 8–32 帧；轨道扫描每旋转 5 度取一帧共 72 帧/圈；路径式采集起点旋转 360 度每 12 度一帧（30 图）加沿途均匀 12 帧</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Qwen2.5-VL-7B 经 SpaceAlign 微调获 +4.8%，而仅用 ScenePick 采样只有 +1.3%；论文指出 VLM 在定量推理上部分场景超人类</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>准确率 / EM（精确匹配）；对 Qwen2.5-VL、InternVL2 等多个基座统一微调后对比</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>huggingface.co/Qwen/Qwen3-VL-8B-Instruct; huggingface.co/Qwen/Qwen3-VL-30B-A3B-Instruct</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3692302</t>
-        </is>
-      </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>★★ 自建 ScanForgeQA 与开源基座（HF 上的 Qwen3-VL）可得；⚠️ 跨方法完整对照表数值需查表</t>
-        </is>
-      </c>
-      <c r="O65" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P65" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q65" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="R65" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S65" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T65" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U65" t="n">
-        <v>63</v>
-      </c>
-      <c r="V65" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W65" t="inlineStr">
-        <is>
-          <t>C004_SpaceEra___ A Unified Framework Towards 3D Spatial Reasoning in Video.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>CoDA: Color Distribution Probing for Efficient and Generalizable AI-Generated Image Detection.</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>FakeForm（自建）· ForenSynths · GenImage</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>FakeForm 约 370,000 图 / 62 个领域；真实图从 COCO/ImageNet/LSUN 等十个公开集随机采 100,000 张；合成图每个生成模型用 HPDv2 提示子集生成 6 万+ 张</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>跨模型（写实内容）平均准确率 91.0%，跨域设定 77.7%（现有检测器域内 &gt;95% 但跨域 &lt;75%）；ForenSynths 上 Acc/AP 98.2/99.6 达 SOTA，超或持平 FatFormer；GenImage 上 95.9% / 99.1% AP 为最佳；跨域均值 77.7/88.1 Acc/AP 超全部对照含大型 VLM；仅 1.48M 参数（对照 AIGI-Holmes 为 7B+）；完整模型将 FakeForm 准确率从单分支的 66.8% 提到 77.7%</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>准确率 Acc、平均精度 AP；分域内/跨模型/跨域三档设定</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3696399</t>
-        </is>
-      </c>
-      <c r="N66" t="inlineStr">
-        <is>
-          <t>★★★ 参数仅 1.48M，复现算力几乎为零；ForenSynths 与 GenImage 公开，自建 FakeForm 规模大且跨域设定最能暴露泛化短板</t>
-        </is>
-      </c>
-      <c r="O66" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P66" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q66" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="R66" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S66" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T66" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U66" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="V66" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W66" t="inlineStr">
-        <is>
-          <t>C005_CoDA_ Color Distribution Probing for Efficient and Generalizable AI-Ge.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>GPT4Point++: Advancing Unified Point-Language Understanding and Generation.</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Objaverse / Objaverse-XL 三级数据 · Cap3D · 3D 点云问答基准</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>Level-1 由 Objaverse-XL 34 万物体与 Objaverse-v1.0 合成 100 万物体（Capverse 严格过滤后保留 4 万高质量，精炼为 70 万）；Level-2 66 万物体（对齐 Cap3D）；Level-3 约 7.9 万物体带密集描述</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>点云描述任务超 VLM 的 InstructBLIP 12.42、超 PointLLM 2.57；3D 点云问答零样本准确率超 InstructBLIP 11.7、超 PointLLM 4.2</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>CIDEr/BLEU/METEOR（描述）、零样本问答准确率；另有 user study 与 GPT4Point 打分的一致性分析（非主判据）</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>github.com/InternLM/InternLM</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3597938</t>
-        </is>
-      </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>★★ Objaverse 系列公开，客观指标齐备；⚠️ 本文 PDF 为 IEEE 早期访问版（作者接收稿），官方排版版尚未发布</t>
-        </is>
-      </c>
-      <c r="O67" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P67" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q67" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="R67" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S67" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T67" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U67" t="n">
-        <v>62.1</v>
-      </c>
-      <c r="V67" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W67" t="inlineStr">
-        <is>
-          <t>C006_GPT4Point___ Advancing Unified Point-Language Understanding and Genera.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>AeroVerse: UAV-Agent Benchmark Suite for Simulating, Pre-training, Finetuning, and Evaluating Aerospace Embodied Foundation Models.</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>AeroVerse 基准套件（AerialAgent-Ego15k · CyberAgent-Ego500k 等五项任务集）</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>AerialAgent-Ego15k 与 CyberAgent-Ego500k 两个自建集；对照参考 ScanNet 1,513 室内场景、EQA 9,000 问答对/774 房间、ALFRED 25,743 指令/428,322 图-动作对</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>SkyAgentX 在四项核心任务（场景感知、空间推理、导航探索、任务规划）上平均超既有方法 8.52%；SkyAgent 在上海场景 BLEU 0.4302 vs Qwen 0.2305、SPICE 0.3083 vs 对照；另一设定 BLEU/SPICE 0.4598/0.3846；人类偏好分 0.87–0.88 远超 GPT-4o 的 0.40–0.45</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>BLEU / SPICE / CIDEr（GPT-4 辅助评分 + 传统文本匹配指标）；另含人类偏好分（补充）</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>github.com/06f081zyd/AeroVerse; huggingface.co/blog/rlhf</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3697634</t>
-        </is>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>★★ 基准套件 GitHub 公开，GPT-4 评分可由 AI 自动化复现；⚠️ 人类偏好分无法自动化，需只取 BLEU/SPICE 口径；PDF 为早期访问版</t>
-        </is>
-      </c>
-      <c r="O68" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P68" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q68" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S68" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T68" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U68" t="n">
-        <v>61.1</v>
-      </c>
-      <c r="V68" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="W68" t="inlineStr">
-        <is>
-          <t>C007_AeroVerse_ UAV-Agent Benchmark Suite for Simulating_ Pre-training_ Fin.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Spherical Vision Transformers for Audio-Visual Saliency Prediction in 360$^{\circ }$∘ Videos.</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Salient360 · PVS-HMEM · VR-EyeTracking · 自建 YT360-EyeTracking</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>PVS-HMEM 含 58 名被试对 76 段 360° 视频的头动与眼动数据；VR-EyeTracking 含 208 段视频（训练 134 / 测试 74），时长 20–60 秒，每段至少 31 人观看、每人看约 35 段</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>⚠️ 未抽到可对比数值：正文称 SalViT360 与 SalViT360-AV 在含自建 YT360-EyeTracking 在内的多个基准上显著超越现有方法，但数值仅存于表格，需人工核表</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>CC（线性相关）、NSS（归一化扫描路径显著性）、AUC-Judd、KLD；真值为眼动仪采集的注视图（采集是人工，但评测本身全自动）</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3604091</t>
-        </is>
-      </c>
-      <c r="N69" t="inlineStr">
-        <is>
-          <t>★★ 三个既有 360° 眼动数据集公开；⚠️ SOTA 数值需查表；自建 YT360-EyeTracking 释出情况未明</t>
-        </is>
-      </c>
-      <c r="O69" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P69" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q69" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="R69" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S69" t="inlineStr">
-        <is>
-          <t>无可对比数值</t>
-        </is>
-      </c>
-      <c r="T69" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U69" t="n">
-        <v>61</v>
-      </c>
-      <c r="V69" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W69" t="inlineStr">
-        <is>
-          <t>C008_Spherical Vision Transformers for Audio-Visual Saliency Prediction in.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Breaking Barriers, Localizing Saliency: A Large-Scale Benchmark and Baseline for Condition-Constrained Salient Object Detection.</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>CSOD10K（自建）· DUTS-TE · DUT-OMRON · PASCAL-S</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>CSOD10K 含 10,000 张高质量真实图，系统覆盖三大约束类型（恶劣环境、介质干扰、成像缺陷）；PASCAL-S 850 图（源自 PASCAL VOC 2010 验证集）</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>CSSAM（Hiera-B 骨干）MAE 0.035 / F-measure 0.887 / S-measure 0.886 / E-measure 0.916，显著超所有 Swin-B 与 ViT-B 骨干方法；CSSAM-L 较同用 SAM 的 MDSAM：MAE −33.3%、F +3.5%、S +3.9%、E +4.0%；DUTS-TE 上较 DCNet MAE +17.4%、F +1.5%；DUT-OMRON 上较 MDSAM MAE +7.7%、S +1.0%；PASCAL-S 上较 TRACER MAE +12.8%、F +1.2%、S +1.7%；仅 42.88M 参数</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>MAE、F-measure、S-measure、E-measure（SOD 标准四件套）；同时报参数量</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3642893</t>
-        </is>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>★★★ 数值完整、对照面广、同时给参数量；DUTS/DUT-OMRON/PASCAL-S 公开；⚠️ 自建 CSOD10K 未见下载链接</t>
-        </is>
-      </c>
-      <c r="O70" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P70" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q70" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="R70" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S70" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T70" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U70" t="n">
-        <v>61</v>
-      </c>
-      <c r="V70" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W70" t="inlineStr">
-        <is>
-          <t>C009_Breaking Barriers_ Localizing Saliency_ A Large-Scale Benchmark and Ba.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Developing Evolving Adaptability in Biological Intelligence: A Novel Biologically-Inspired Continual Learning Model for Video Saliency Prediction.</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>DHF1K · Hollywood-2 · UCF Sports</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>DHF1K 1,000 段视频；Hollywood-2 1,707 段（来自 69 部电影、12 类动作）；UCF Sports 150 段 9 类</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>⚠️ 未抽到跨方法数值：正文只给出本模型的效率画像（约 8.8 GFLOPs、52 FPS、模型 42.35 MB）与"在三个基准上定量定性均超近期 SOTA"的定性结论，具体对照数值需人工核表</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>CC、NSS、AUC-Judd、SIM、s-AUC（视频显著性预测标准指标）；同时报 GFLOPs/FPS/模型体积</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3643517</t>
-        </is>
-      </c>
-      <c r="N71" t="inlineStr">
-        <is>
-          <t>★★ DHF1K/Hollywood-2/UCF Sports 为该领域三大公开基准，指标客观；⚠️ SOTA 数值需查表，未见代码链接</t>
-        </is>
-      </c>
-      <c r="O71" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P71" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q71" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="R71" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S71" t="inlineStr">
-        <is>
-          <t>无可对比数值</t>
-        </is>
-      </c>
-      <c r="T71" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U71" t="n">
-        <v>61</v>
-      </c>
-      <c r="V71" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W71" t="inlineStr">
-        <is>
-          <t>C010_Developing Evolving Adaptability in Biological Intelligence_ A Novel B.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>On Structuring Hyperspherical Manifold for Probing Novel Biomedical Entities.</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>新类发现与定位基准（含 COVID-19 影像集等生物医学实体数据）</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>覆盖多个生物医学实体识别与新类发现设定</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>⚠️ 数值不完整：正文以"灰色列代表未见实体的类别归属正确率，本文的几何约束处理超过次优对照"表述，未给绝对数值；对照含 RankStats+ 等一众新类发现方法</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>未见类别的分配正确率、聚类准确率；新类发现标准评测协议</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3596597</t>
-        </is>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>★★ 对照面广、指标客观；⚠️ 论文未给可直接引用的数值，接入前需查表；未见代码与数据链接</t>
-        </is>
-      </c>
-      <c r="O72" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P72" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q72" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="R72" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S72" t="inlineStr">
-        <is>
-          <t>无可对比数值</t>
-        </is>
-      </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U72" t="n">
-        <v>60.9</v>
-      </c>
-      <c r="V72" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W72" t="inlineStr">
-        <is>
-          <t>C011_On Structuring Hyperspherical Manifold for Probing Novel Biomedical En.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Alliance: All-in-One Spectral-Spatial-Frequency Awareness Foundation Model.</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>BigEarthNet 类多标签分类 · OSCD 变化检测 · QUH-Pingan · QUH-Tangdaowan · 域间分割</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>官方划分 14 对训练 / 10 对验证；QUH-Pingan 176 波段 1230×1000 共 10 类；QUH-Tangdaowan 176 波段 1740×860 共 18 类；两者每类取 100 点训练、其余验证</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>多标签分类 micro-mAP 88.59% / macro-mAP 88.67%，超最佳基座 SatMAE++ 1.18% 与 0.92%；OSCD 变化检测 F1 56.87%，超最佳变化检测模型 ChangeFormer(54.72%) 2.15%、超最佳基座 SpectralGPT+(54.30%) 2.57%；域间分割 mIoU 67.20%，超最佳域适应方法 CLAN(65.62%) 1.58%、超最佳域泛化方法 VisualDG(64.97%) 2.23%；消融链 65.52%→65.67%→67.20%</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>micro/macro-mAP、F1、mIoU；分多标签分类、变化检测、域间分割三类任务</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3639595</t>
-        </is>
-      </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>★★★ 数值完整且三类任务分别对标各自最强基线，OSCD 与 QUH 系列公开；⚠️ 未见代码链接</t>
-        </is>
-      </c>
-      <c r="O73" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P73" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q73" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="R73" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S73" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T73" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U73" t="n">
-        <v>59</v>
-      </c>
-      <c r="V73" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W73" t="inlineStr">
-        <is>
-          <t>C012_Alliance_ All-in-One Spectral-Spatial-Frequency Awareness Foundation M.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Learning Compact Semantic Information and Reliable Pseudo-Labels for Incomplete Multi-View Multi-Label Classification.</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>Corel5k · Pascal07 · ESPGame · IAPRTC-12 · Mirflickr 等七个多视图多标签集</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Pascal07 9,963 图；ESPGame 20,7xx 图（平均每图 4.69 个标签）；IAPRTC-12 近 20,000 图 291 个标签；Mirflickr 25,000 图</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>在七个数据集、视图与标签双缺失率 30%/50% 及完整数据三种设定下，均优于十种 SOTA 方法；具体 AP 数值在表格中，另有 λ1/λ2 与 τu/τb 的敏感性曲线</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>AP（平均精度）；按视图缺失率 κv 与标签缺失率 κl 分档</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3665813</t>
-        </is>
-      </c>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>★★ 五个多标签数据集均为公开标准集，双缺失率设定明确；⚠️ 逐数据集 AP 需查表，未见代码链接</t>
-        </is>
-      </c>
-      <c r="O74" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P74" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q74" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="R74" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S74" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T74" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U74" t="n">
-        <v>59</v>
-      </c>
-      <c r="V74" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W74" t="inlineStr">
-        <is>
-          <t>C013_Learning Compact Semantic Information and Reliable Pseudo-Labels for I.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Foundation Models based Scene Graph Generation.</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>基因组与序列</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>Visual Genome VG150 · GQA</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>VG150 含 150 个物体类与 50 种关系类；三种评测模式 PredCls / SGCls / SGDet</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>VG150 上 mR@100 为 39.4(PredCls)/26.6(SGCls)/22.2(SGDet)；mR@50 达 46.5% 超全部对照；较 VCTree+ST-SGG 在三模式上 +3.8%/4.2%/6.1%；较 MotifsNet+TBE +11.1%/8.6%/10.2%；按 AVG zR 计三模式分别超全部基线 6.2%–19.0% / 4.9%–9.3% / 3.6%–6.4%；GQA 上 mR@100 较 Transformer+CFA +11.4%/4.4%/4.1%；对照的去偏方法 TransRwt/PPDL/CFA 在 PredCls 下 R@100 反而下降 18.2%/20.1%/10.9%，本方法无此代价</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>R@K、mR@K（均值召回）、zR@K（零样本召回）；PredCls/SGCls/SGDet 三种标准评测模式</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3712094</t>
-        </is>
-      </c>
-      <c r="N75" t="inlineStr">
-        <is>
-          <t>★★★ VG150 与 GQA 为场景图领域标准集，三模式评测协议成熟；论文点出去偏方法牺牲 R@100 的通病，对设基线很有价值；⚠️ 未见代码链接</t>
-        </is>
-      </c>
-      <c r="O75" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P75" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q75" t="inlineStr">
-        <is>
-          <t>基因组与序列</t>
-        </is>
-      </c>
-      <c r="R75" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S75" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T75" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U75" t="n">
-        <v>59</v>
-      </c>
-      <c r="V75" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W75" t="inlineStr">
-        <is>
-          <t>C014_Foundation Models based Scene Graph Generation.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Efficient Heterogeneous Exploration with Mutual Policy Divergence Maximization for Multiagent Reinforcement Learning.</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>推荐与信息检索</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>MA-MuJoCo（9 个任务）· Bi-DexHands（8 个任务）· Google Research Football（8 个任务）</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>三个基准共 25 个异构场景</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>正文称在 25 个异构场景上一致超越现有 SOTA 序贯更新类方法；训练开销较 A2PO 增加 7.9%–11.1%；⚠️ 逐任务回报/胜率数值在表格与曲线中</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>回合回报、胜率；同时报训练时间开销</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3718850</t>
-        </is>
-      </c>
-      <c r="N76" t="inlineStr">
-        <is>
-          <t>★★ 三个 MARL 基准全部公开且环境标准化，指标客观可自动化；⚠️ 跨方法数值需查表，未见代码链接；PDF 为 IEEE 早期访问版</t>
-        </is>
-      </c>
-      <c r="O76" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P76" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q76" t="inlineStr">
-        <is>
-          <t>推荐与信息检索</t>
-        </is>
-      </c>
-      <c r="R76" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S76" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T76" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U76" t="n">
-        <v>59</v>
-      </c>
-      <c r="V76" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W76" t="inlineStr">
-        <is>
-          <t>C015_Efficient Heterogeneous Exploration with Mutual Policy Divergence Maxi.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>76</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Feature-Space Planes Searcher: A Universal Domain Adaptation Framework for Interpretability and Computational Efficiency.</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>推荐与信息检索</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>DomainNet · Office-Home 等通用域适应基准</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>ResNet 与 ViT 两类骨干；源域准确率引自原论文</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>⚠️ 未抽到可对比数值：正文以 PAC-Bayes 框架给理论分析，实验数值（含"有无特征几何退化"的消融，原设定 α=β=1.0）全在表格中，未被文本层解析</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>目标域分类准确率、H-score；通用域适应（UniDA）标准协议</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3703974</t>
-        </is>
-      </c>
-      <c r="N77" t="inlineStr">
-        <is>
-          <t>★★ DomainNet/Office-Home 公开；⚠️ SOTA 数值需人工核表，未见代码链接</t>
-        </is>
-      </c>
-      <c r="O77" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P77" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q77" t="inlineStr">
-        <is>
-          <t>推荐与信息检索</t>
-        </is>
-      </c>
-      <c r="R77" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S77" t="inlineStr">
-        <is>
-          <t>无可对比数值</t>
-        </is>
-      </c>
-      <c r="T77" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U77" t="n">
-        <v>58.9</v>
-      </c>
-      <c r="V77" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W77" t="inlineStr">
-        <is>
-          <t>C016_Feature-Space Planes Searcher_ A Universal Domain Adaptation Framework.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>A Natural Language Guided Approach for Blind Face Restoration: Methodology and Dataset.</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>自建文本-人脸配对数据集 · CelebA-HQ 等盲脸复原基准</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>用多模态大模型为每张高质图生成文本描述，得 30,000 组文本-图像配对样本</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>FaceCLIP 对齐准确率 93%，匹配/非匹配对相似度分离清晰（18.5 vs 5.37），而 LongCLIP 几乎无区分度（20.55 vs 20.88，另一组 21.86 vs 20.02）；PSNR 上 MultiScaleAtten 略高（25.021 vs 25.016），但本文 TGHAB 在语义忠实度与身份一致性上更优</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>PSNR / SSIM / LPIPS / FID（复原质量）、身份一致性、文本-图像对齐准确率</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>github.com/wcy-cs/TBFR</t>
-        </is>
-      </c>
-      <c r="M78" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3665736</t>
-        </is>
-      </c>
-      <c r="N78" t="inlineStr">
-        <is>
-          <t>★★ 代码承诺公开（wcy-cs/TBFR）；⚠️ 论文自陈 PSNR 略逊于对照，主要优势在语义与身份维度，选基线时需注意口径</t>
-        </is>
-      </c>
-      <c r="O78" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P78" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q78" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S78" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T78" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U78" t="n">
-        <v>58.7</v>
-      </c>
-      <c r="V78" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W78" t="inlineStr">
-        <is>
-          <t>C017_A Natural Language Guided Approach for Blind Face Restoration_ Methodo.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>ChatTracker: Enhancing Visual Tracking via LLM-Driven Iterative Description Refinement.</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>LaSOT · LaSOText · TNL2K 等视觉跟踪基准</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>LaSOT 为大规模长时跟踪集；无公开预训练权重的对照方法直接引用其论文数值</t>
-        </is>
-      </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>某基准 AUC 74.1%，超 JointNLT 达 13.7%；另一挑战集上 ChatTracker-L AUC 86.1% 超此前全部跟踪器；LaSOText 上 AUC 56.1% 超 UVLTrack；较 UVLTrack-L 在 AUC 上 +0.64%；精确率较 JointNLT +12.4%；生成描述的错误率仅 6.61%，比数据集原始人工标注描述低 7.3 个百分点</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>AUC、精确率 P、归一化精确率 Pnorm；描述不准确率（Inaccuracy Ratio）</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3674357</t>
-        </is>
-      </c>
-      <c r="N79" t="inlineStr">
-        <is>
-          <t>★★★ LaSOT 系列公开且有标准评测工具；论文用"生成描述比人工标注更准"这一点很有意思；⚠️ 未见代码链接</t>
-        </is>
-      </c>
-      <c r="O79" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P79" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q79" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="R79" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S79" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T79" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U79" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="V79" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W79" t="inlineStr">
-        <is>
-          <t>C018_ChatTracker_ Enhancing Visual Tracking via LLM-Driven Iterative Descri.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>OmniCharacter++: Toward Comprehensive Benchmark for Realistic Role-Playing Agents.</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>LLM与agent</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>OmniCharacter++（自建角色扮演基准）</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>训练集 88,474 段双人对话（平均 10.00 轮）+ 29,543 段多角色对话（平均 15.05 轮），共 118,017 段；人工抽检 100 条测试样本校准 GPT-4o 评分</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>UniCharacter（7B）在所有裁判模型下全指标最优，超 GPT-4、Gemini-2.0-flash；OmniCharacter 多数设定下排第二，超 GPT-3.5、Doubao-1.5-Pro、Qwen2.5-7B-Instruct；完整组件达 51.81% / 2.57；平均分 3.304，超 MiniMax +0.170、超 InternLM-20B +0.181（自身仅 7B）；带音频版角色一致性 3.102、对话能力 3.612（去音频为 3.015）；双人对话情感维度 6.94 vs 6.61/6.65</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>多维度 LLM-as-judge 打分（角色一致性、对话能力、情感等），基座为 Qwen2.5-7B-Instruct；另有 100 条人工抽检用于校准裁判偏差</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>github.com/zchoi/OmniCharacter-</t>
-        </is>
-      </c>
-      <c r="M80" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3690447</t>
-        </is>
-      </c>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>★★★ 代码与基准公开（zchoi/OmniCharacter-plus），主判据 GPT-4o 打分可由 AI 完整复现；人工抽检仅用于校准，不阻断自动化</t>
-        </is>
-      </c>
-      <c r="O80" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P80" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q80" t="inlineStr">
-        <is>
-          <t>LLM与agent</t>
-        </is>
-      </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S80" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T80" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U80" t="n">
-        <v>57.9</v>
-      </c>
-      <c r="V80" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="W80" t="inlineStr">
-        <is>
-          <t>C019_OmniCharacter___ Toward Comprehensive Benchmark for Realistic Role-Pla.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Brightness-Aware Synthetic-to-Real Learning for Nighttime Hazy Image Enhancement.</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>真实夜间雾天测试集（150 图）· 合成夜间雾天数据</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>测试用 150 张真实世界图；对照方法含 MRP、GD、OSFD、MSBDN 等</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>一组设定下 SSIM 0.966 / PSNR 34.254，超次优的 0.953 / 33.291；另一组 SSIM 0.898 / PSNR 29.807，超次优的 0.868 / 28.854</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>PSNR / SSIM；分合成数据与真实数据两套对照</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>github.com/Xiaofeng-life/SFN</t>
-        </is>
-      </c>
-      <c r="M81" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3671754</t>
-        </is>
-      </c>
-      <c r="N81" t="inlineStr">
-        <is>
-          <t>★★★ 代码承诺公开（Xiaofeng-life/SFN），PSNR/SSIM 客观；⚠️ 150 张真实测试图的来源集需向作者确认可得性</t>
-        </is>
-      </c>
-      <c r="O81" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P81" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q81" t="inlineStr">
-        <is>
-          <t>视觉-分割检测</t>
-        </is>
-      </c>
-      <c r="R81" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S81" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T81" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U81" t="n">
-        <v>57.6</v>
-      </c>
-      <c r="V81" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W81" t="inlineStr">
-        <is>
-          <t>C020_Brightness-Aware Synthetic-to-Real Learning for Nighttime Hazy Image E.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Communication-Efficient Federated Multi-View Clustering.</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>表格与通用ML</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>ORL · Flower17 等多视图聚类标准集</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>Flower17 为 17 类每类 80 图；参数 λ 与 β 在 2^-10 到 2^10 范围扫描</t>
-        </is>
-      </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>较现有联邦多视图聚类方法：平均准确率 +26.84%、计算加速 2.9×–2153×、通信开销最多降 98.4%；较次优方法 ACC/NMI/purity 分别 +5.24%/+2.26%/+3.51%</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>ACC、NMI、purity；同时报计算加速比与通信开销；所有对照方法直接跑作者官网公开代码、不做改动</t>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3601533</t>
-        </is>
-      </c>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>★★★ 明确说明对照方法用官方代码原样复跑，这是本批公平性做得最扎实的一篇；ORL/Flower17 公开</t>
-        </is>
-      </c>
-      <c r="O82" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P82" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q82" t="inlineStr">
-        <is>
-          <t>表格与通用ML</t>
-        </is>
-      </c>
-      <c r="R82" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S82" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T82" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U82" t="n">
-        <v>57</v>
-      </c>
-      <c r="V82" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W82" t="inlineStr">
-        <is>
-          <t>C021_Communication-Efficient Federated Multi-View Clustering.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Robust Semi-Supervised Feature Selection With Multi-Granularity Zentropy Modeling.</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>表格与通用ML</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>16 个特征选择基准数据集（记为 D1–D16）</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>16 个数据集；标签缺失比例从 0 到 60% 共九档</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>九种缺失比例下分别在 12/11/11/11/11/11/14/13/15 个数据集上胜过基线；16 个数据集中 13 次取得最高均值；缺失率升到 60% 时仍在 13 与 14 个数据集上最优；20% 缺失时除 D13 在分类器 C2 上外全面超 FSZE；40% 缺失时 Inf-FS/FScNCE/FSZE 分别只在 10/4/2 个数据集上取得最少特征数</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>分类准确率（多个下游分类器）、所选特征数；用 Friedman 检验加临界差 CD（M=10, D=16 时 CD=3.1257）做统计显著性</t>
-        </is>
-      </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3647921</t>
-        </is>
-      </c>
-      <c r="N83" t="inlineStr">
-        <is>
-          <t>★★ 带完整统计检验，评测严谨；⚠️ 论文以"在 N 个数据集上胜出"的计数式表述为主，绝对数值需查表；未见代码与数据链接</t>
-        </is>
-      </c>
-      <c r="O83" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P83" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q83" t="inlineStr">
-        <is>
-          <t>表格与通用ML</t>
-        </is>
-      </c>
-      <c r="R83" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S83" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T83" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U83" t="n">
-        <v>57</v>
-      </c>
-      <c r="V83" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W83" t="inlineStr">
-        <is>
-          <t>C022_Robust Semi-Supervised Feature Selection With Multi-Granularity Zentro.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>MRCNet: Motion Reasoning Chain for Cross Modal Video Camouflaged Object Detection.</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>MoCA-Mask · CAD2016 · COD10K（预训练）</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>MoCA-Mask 87 段视频共 22,939 帧（训练 71 段 / 测试 16 段）；CAD2016 2,600 帧带像素级掩码；先在 COD10K 预训练再于 MoCA-Mask 微调</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>MoCA-Mask 上 mDice 超 ZoomNext 5.9%、超基于提示学习的 TSP-SAM 9.8%</t>
-        </is>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>mDice、mIoU、MAE、S-measure，以及时序连续性 TC(t) 与空间一致性 SC(t) 两个时空指标</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3689767</t>
-        </is>
-      </c>
-      <c r="N84" t="inlineStr">
-        <is>
-          <t>★★★ MoCA-Mask/CAD2016/COD10K 全公开，预训练-微调流程明确；额外的时空一致性指标对视频任务评测有参考价值；⚠️ 未见代码链接</t>
-        </is>
-      </c>
-      <c r="O84" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P84" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q84" t="inlineStr">
-        <is>
-          <t>视觉-视频与具身</t>
-        </is>
-      </c>
-      <c r="R84" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S84" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T84" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U84" t="n">
-        <v>57</v>
-      </c>
-      <c r="V84" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W84" t="inlineStr">
-        <is>
-          <t>C023_MRCNet_ Motion Reasoning Chain for Cross Modal Video Camouflaged Objec.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Partial Contrastive Learning for Partially View-aligned Multi-view Clustering.</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Deep Caltech-101 · Scene-15 · WIKI · CUB-200-2011 等八个多视图基准</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>Deep Caltech-101 8,677 图 101 类；Scene-15 4,485 图 15 类；WIKI 2,866 组图文对 10 类；对齐比例 ς=0.5</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>在八个基准上与十一个有竞争力的基线做定量对比（Table I，ς=0.5），全设定下一致超越；LPCL 优于标准 InfoNCE</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>ACC、NMI、purity；按视图对齐比例 ς 分档</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3694999</t>
-        </is>
-      </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>★★ 八个多视图数据集均为公开标准集；⚠️ 逐数据集数值在表格中；PDF 为 IEEE 早期访问版，未见代码链接</t>
-        </is>
-      </c>
-      <c r="O85" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P85" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q85" t="inlineStr">
-        <is>
-          <t>其他</t>
-        </is>
-      </c>
-      <c r="R85" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S85" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T85" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U85" t="n">
-        <v>57</v>
-      </c>
-      <c r="V85" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W85" t="inlineStr">
-        <is>
-          <t>C024_Partial Contrastive Learning for Partially View-aligned Multi-view Clu.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="n">
-        <v>85</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>DEMO-EMol: modeling protein-nucleic acid complex structures from cryo-EM maps by coupling chain assembly with map segmentation.</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Nucleic Acids Research</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>蛋白与结构</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>自建 cryo-EM 基准：49 个蛋白-核酸复合物 + 48 个蛋白-蛋白复合物</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>分辨率跨度 1.96–12.77 Å（另一子集 2.41 Å 起）；链拟合以相关系数 0.6 为阈值</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>平均 TM-score 0.92，较 DiffModeler(0.83) 高 10.8%、较 Phenix(0.76) 高 21.1%；另一设定平均 TM-score 0.91，较 DiffModeler(0.80)/Phenix(0.70)/EMBuild(0.84) 高 13.8%/30.0%/8.3%；平均 RMSD 4.8 Å，优于 DiffModeler(11.2 Å)、Phenix(16.1 Å)、EMBuild(6.3 Å)；以 AlphaFold3 链模型(TM 0.88)起步可达 TM 0.96 / RMSD 4.7 Å，而 DiffModeler 为 0.72 / 8.0 Å；t 检验 p 值 5.61e-4、4.18e-5、2.48e-1</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>TM-score、RMSD（Å）、链相关系数；Student's t 检验报显著性</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1093/nar/gkaf416</t>
-        </is>
-      </c>
-      <c r="N86" t="inlineStr">
-        <is>
-          <t>★★★ 数值最完整的生信类之一，对照 DiffModeler/Phenix/EMBuild/AlphaFold3 且带统计检验；cryo-EM 图谱可从 EMDB 公开下载；⚠️ 基准清单在 Supplementary，需一并取</t>
-        </is>
-      </c>
-      <c r="O86" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="P86" t="inlineStr">
-        <is>
-          <t>生信</t>
-        </is>
-      </c>
-      <c r="Q86" t="inlineStr">
-        <is>
-          <t>蛋白与结构</t>
-        </is>
-      </c>
-      <c r="R86" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S86" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T86" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U86" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="V86" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W86" t="inlineStr">
-        <is>
-          <t>C025_DEMO-EMol_ modeling protein-nucleic acid complex structures from cryo-.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Stereo-Talker: Audio-driven 3D Human Synthesis with Prior-Guided Mixture-of-Experts.</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>时序与信号</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>HDTF · TikTok · MVHumanNet（各取 10 段作测试集）· 自采数据集</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>自采 3,425 段网络视频 + 1,325 段来自既有数据集；验证集随机 100 段、测试集另 200 段；三个公开数据集各取 10 段分别用于视频生成与说话头生成</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>HDTF 说话头：本方法 7.17/7.93/17.36/0.058/0.591，对照 SadTalker 22.36/0.124/0.752、Aniportrait 3.51/11.11/32.86/0.225/0.641（FID 17.36 vs 32.86）；视角可控人体视频生成（Table 6，LVD↓/L1↓/Diversity↑）：本方法 0.031/0.034/1.721，SHOW 0.029/0.072/0.356，Diffgesture 0.065/0.076/1.150，真值 0/0/2.201；对照 Human4dit 1333.73/3.100/99.78/0.187/1.234 vs 本方法 747.70/2.603/68.73/0.196/1.193；主观分（Table 3，1–5 分）Vlogger 1.88/2.2/2.44/2.68 vs 本方法 4.02/3.5/4.46/4.1</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>客观：LVD（顶点距离）、L1、Diversity、FID、FVD、LPIPS、LSE-C/LSE-D（唇同步）；主观：Diversity/Synchrony/Clarity/Overall Quality 各 1–5 分（仅作补充）</t>
-        </is>
-      </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>github.com/Breakthrough/PySceneDetect; github.com/Zulko/moviepy</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2025.3596160</t>
-        </is>
-      </c>
-      <c r="N87" t="inlineStr">
-        <is>
-          <t>★★ 测试集取自公开的 HDTF/TikTok/MVHumanNet，客观指标数值完整可对照；⚠️ 训练集为自采网络视频不公开，论文明言"不存在同时满足身份数、音视频同步、多视角条件的公开数据集"；主表含主观评分，复现时应只取客观口径</t>
-        </is>
-      </c>
-      <c r="O87" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P87" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q87" t="inlineStr">
-        <is>
-          <t>时序与信号</t>
-        </is>
-      </c>
-      <c r="R87" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S87" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T87" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U87" t="n">
-        <v>46</v>
-      </c>
-      <c r="V87" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W87" t="inlineStr">
-        <is>
-          <t>C026_Stereo-Talker_ Audio-driven 3D Human Synthesis with Prior-Guided Mixtu.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>When 'Yes' Meets 'But': Can AI Comprehend Contradictory Humor in Comics?</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>IEEE Trans. Pattern Analysis and Machine Intelligence</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>LLM与agent</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>YES-BUT（自建，由 349 图扩至 1,262 图）</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>1,262 张漫画；其中 257 张含中文文本、113 张含英文文本；人工评估仅抽 30 条样本作为补充</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>LLaVA-OneVision 系列一致超 LLaVA-1.5 与 LLaVA-Next；同参数量下 LLaVA-Next 一致超 LLaVA-1.5；商用模型在字面描述生成上普遍优于开源模型；⚠️ 逐模型绝对分数在表格中</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>选择题准确率与 F1（客观部分）；字面/深层描述生成用 ROUGE 与 LLM-as-judge；30 条人工评估仅作补充</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1109/tpami.2026.3688191</t>
-        </is>
-      </c>
-      <c r="N88" t="inlineStr">
-        <is>
-          <t>★★ 基准自建且规模明确，客观题部分完全可自动化；⚠️ 生成部分依赖 LLM 裁判，绝对数值需查表，未见数据集下载链接</t>
-        </is>
-      </c>
-      <c r="O88" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="P88" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="Q88" t="inlineStr">
-        <is>
-          <t>LLM与agent</t>
-        </is>
-      </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>原创方法</t>
-        </is>
-      </c>
-      <c r="S88" t="inlineStr">
-        <is>
-          <t>完整</t>
-        </is>
-      </c>
-      <c r="T88" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="U88" t="n">
-        <v>43.1</v>
-      </c>
-      <c r="V88" t="inlineStr">
-        <is>
-          <t>部分</t>
-        </is>
-      </c>
-      <c r="W88" t="inlineStr">
-        <is>
-          <t>C027_When _Yes_ Meets _But__ Can AI Comprehend Contradictory Humor in Comic.pdf</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:W88"/>
+  <autoFilter ref="A1:W61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>